<commit_message>
highlighted filed_data columns w.ref of HT form
</commit_message>
<xml_diff>
--- a/AzamSb/16Jul26/PESCO Combined HT and LT Sample Data files received by PESCO, 09JUNE2026/HAYATABAD-2/Lat long toXY conversion New.xlsx
+++ b/AzamSb/16Jul26/PESCO Combined HT and LT Sample Data files received by PESCO, 09JUNE2026/HAYATABAD-2/Lat long toXY conversion New.xlsx
@@ -677,7 +677,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -727,40 +727,31 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="5" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1084,12 +1075,12 @@
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="B4" s="25" t="s">
+      <c r="B4" s="35" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="26"/>
-      <c r="D4" s="26"/>
-      <c r="E4" s="26"/>
+      <c r="C4" s="36"/>
+      <c r="D4" s="36"/>
+      <c r="E4" s="36"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B5" s="4" t="s">
@@ -1109,7 +1100,7 @@
       <c r="B6" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="31">
+      <c r="C6" s="25">
         <v>33.996749999999999</v>
       </c>
       <c r="D6" s="6" t="s">
@@ -1123,7 +1114,7 @@
       <c r="B7" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="32">
+      <c r="C7" s="26">
         <v>71.440866</v>
       </c>
       <c r="D7" s="6" t="s">
@@ -1134,12 +1125,12 @@
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="B9" s="25" t="s">
+      <c r="B9" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="26"/>
-      <c r="D9" s="26"/>
-      <c r="E9" s="26"/>
+      <c r="C9" s="36"/>
+      <c r="D9" s="36"/>
+      <c r="E9" s="36"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B10" s="4" t="s">
@@ -1159,7 +1150,7 @@
       <c r="B11" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="30">
+      <c r="C11" s="8">
         <f>INT((C7+180)/6)+1</f>
         <v>42</v>
       </c>
@@ -1174,7 +1165,7 @@
       <c r="B12" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="30">
+      <c r="C12" s="8">
         <f>(C11*6)-183</f>
         <v>69</v>
       </c>
@@ -1257,12 +1248,12 @@
       </c>
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B19" s="25" t="s">
+      <c r="B19" s="35" t="s">
         <v>36</v>
       </c>
-      <c r="C19" s="26"/>
-      <c r="D19" s="26"/>
-      <c r="E19" s="26"/>
+      <c r="C19" s="36"/>
+      <c r="D19" s="36"/>
+      <c r="E19" s="36"/>
     </row>
     <row r="20" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B20" s="4" t="s">
@@ -1423,12 +1414,12 @@
       </c>
     </row>
     <row r="31" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B31" s="25" t="s">
+      <c r="B31" s="35" t="s">
         <v>58</v>
       </c>
-      <c r="C31" s="26"/>
-      <c r="D31" s="26"/>
-      <c r="E31" s="26"/>
+      <c r="C31" s="36"/>
+      <c r="D31" s="36"/>
+      <c r="E31" s="36"/>
     </row>
     <row r="32" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B32" s="4" t="s">
@@ -1448,7 +1439,7 @@
       <c r="B33" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="C33" s="33">
+      <c r="C33" s="27">
         <f>C16 + C15*C25*(C28 + (1-C26+C27)*(C28^3)/6 + (5-18*C26+C26^2+72*C27-58*C24)*(C28^5)/120)</f>
         <v>725443.02518260828</v>
       </c>
@@ -1465,7 +1456,7 @@
       <c r="B34" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="C34" s="33">
+      <c r="C34" s="27">
         <f>C17 + C15*(C29 + C25*TAN(C21)*((C28^2)/2 + (5-C26+9*C27+4*(C27^2))*(C28^4)/24 + (61-58*C26+C26^2+600*C27-330*C24)*(C28^6)/720))</f>
         <v>3764481.6522049154</v>
       </c>
@@ -1563,11 +1554,11 @@
         <f t="shared" ref="F5:F14" si="1">(E5*6)-183</f>
         <v>69</v>
       </c>
-      <c r="G5" s="34">
+      <c r="G5" s="28">
         <f t="shared" ref="G5:G14" si="2">500000 + 0.9996 * (6378137/SQRT(1-0.00669438*(SIN(RADIANS(C5))^2))) * ((RADIANS(D5-F5)*COS(RADIANS(C5))) + (1 - TAN(RADIANS(C5))^2 + 0.0067395*(COS(RADIANS(C5))^2)) * ((RADIANS(D5-F5)*COS(RADIANS(C5)))^3)/6 + (5 - 18*TAN(RADIANS(C5))^2 + TAN(RADIANS(C5))^4 + 72*0.0067395*(COS(RADIANS(C5))^2) - 58*0.0067395) * ((RADIANS(D5-F5)*COS(RADIANS(C5)))^5)/120)</f>
         <v>725373.50020119664</v>
       </c>
-      <c r="H5" s="34">
+      <c r="H5" s="28">
         <f t="shared" ref="H5:H14" si="3">0.9996 * ((6378137*(0.9983242984*RADIANS(C5) - 0.002514607*SIN(2*RADIANS(C5)) + 0.000002639*SIN(4*RADIANS(C5)) - 0.000000003*SIN(6*RADIANS(C5)))) + (6378137/SQRT(1-0.00669438*(SIN(RADIANS(C5))^2))) * TAN(RADIANS(C5)) * (((RADIANS(D5-F5)*COS(RADIANS(C5)))^2)/2 + (5 - TAN(RADIANS(C5))^2 + 9*0.0067395*(COS(RADIANS(C5))^2) + 4*(0.0067395*(COS(RADIANS(C5))^2))^2) * ((RADIANS(D5-F5)*COS(RADIANS(C5)))^4)/24 + (61 - 58*TAN(RADIANS(C5))^2 + TAN(RADIANS(C5))^4 + 600*0.0067395*(COS(RADIANS(C5))^2) - 330*0.0067395) * ((RADIANS(D5-F5)*COS(RADIANS(C5)))^6)/720))</f>
         <v>3764486.0991854998</v>
       </c>
@@ -1597,11 +1588,11 @@
         <f t="shared" si="1"/>
         <v>75</v>
       </c>
-      <c r="G6" s="34">
+      <c r="G6" s="28">
         <f t="shared" si="2"/>
         <v>319048.64709274552</v>
       </c>
-      <c r="H6" s="34">
+      <c r="H6" s="28">
         <f t="shared" si="3"/>
         <v>3728876.2682867674</v>
       </c>
@@ -1631,11 +1622,11 @@
         <f t="shared" si="1"/>
         <v>75</v>
       </c>
-      <c r="G7" s="34">
+      <c r="G7" s="28">
         <f t="shared" si="2"/>
         <v>439116.47001927451</v>
       </c>
-      <c r="H7" s="34">
+      <c r="H7" s="28">
         <f t="shared" si="3"/>
         <v>3487452.4577139197</v>
       </c>
@@ -1665,11 +1656,11 @@
         <f t="shared" si="1"/>
         <v>69</v>
       </c>
-      <c r="G8" s="34">
+      <c r="G8" s="28">
         <f t="shared" si="2"/>
         <v>298038.08371635771</v>
       </c>
-      <c r="H8" s="34">
+      <c r="H8" s="28">
         <f t="shared" si="3"/>
         <v>2751004.9055434382</v>
       </c>
@@ -1699,11 +1690,11 @@
         <f t="shared" si="1"/>
         <v>69</v>
       </c>
-      <c r="G9" s="34">
+      <c r="G9" s="28">
         <f t="shared" si="2"/>
         <v>305026.24745018093</v>
       </c>
-      <c r="H9" s="34">
+      <c r="H9" s="28">
         <f t="shared" si="3"/>
         <v>3340441.4669071855</v>
       </c>
@@ -1733,11 +1724,11 @@
         <f t="shared" si="1"/>
         <v>63</v>
       </c>
-      <c r="G10" s="34">
+      <c r="G10" s="28">
         <f t="shared" si="2"/>
         <v>431992.448970236</v>
       </c>
-      <c r="H10" s="34">
+      <c r="H10" s="28">
         <f t="shared" si="3"/>
         <v>2778582.4282347457</v>
       </c>
@@ -1767,11 +1758,11 @@
         <f t="shared" si="1"/>
         <v>69</v>
       </c>
-      <c r="G11" s="34">
+      <c r="G11" s="28">
         <f t="shared" si="2"/>
         <v>743174.56404579303</v>
       </c>
-      <c r="H11" s="34">
+      <c r="H11" s="28">
         <f t="shared" si="3"/>
         <v>3338930.7251546346</v>
       </c>
@@ -1801,11 +1792,11 @@
         <f t="shared" si="1"/>
         <v>75</v>
       </c>
-      <c r="G12" s="34">
+      <c r="G12" s="28">
         <f t="shared" si="2"/>
         <v>322783.74721808889</v>
       </c>
-      <c r="H12" s="34">
+      <c r="H12" s="28">
         <f t="shared" si="3"/>
         <v>3481024.5190451923</v>
       </c>
@@ -1835,11 +1826,11 @@
         <f t="shared" si="1"/>
         <v>69</v>
       </c>
-      <c r="G13" s="39">
+      <c r="G13" s="32">
         <f t="shared" si="2"/>
         <v>435404.17311818898</v>
       </c>
-      <c r="H13" s="39">
+      <c r="H13" s="32">
         <f t="shared" si="3"/>
         <v>2808952.6974581978</v>
       </c>
@@ -1865,1021 +1856,1021 @@
         <f t="shared" si="0"/>
         <v>43</v>
       </c>
-      <c r="F14" s="41">
+      <c r="F14" s="30">
         <f t="shared" si="1"/>
         <v>75</v>
       </c>
-      <c r="G14" s="40">
+      <c r="G14" s="33">
         <f t="shared" si="2"/>
         <v>437568.90626172855</v>
       </c>
-      <c r="H14" s="40">
+      <c r="H14" s="33">
         <f t="shared" si="3"/>
         <v>3975385.2584199412</v>
       </c>
-      <c r="I14" s="38" t="str">
+      <c r="I14" s="31" t="str">
         <f t="shared" si="4"/>
         <v>UTM Zone 43N / 437,569E, 3,975,385N</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="C15" s="35"/>
-      <c r="D15" s="35"/>
-      <c r="E15" s="36"/>
-      <c r="F15" s="37"/>
-      <c r="G15" s="42"/>
-      <c r="H15" s="42"/>
-      <c r="I15" s="38"/>
+      <c r="C15" s="29"/>
+      <c r="D15" s="29"/>
+      <c r="E15" s="21"/>
+      <c r="F15" s="30"/>
+      <c r="G15" s="34"/>
+      <c r="H15" s="34"/>
+      <c r="I15" s="31"/>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="C16" s="35"/>
-      <c r="D16" s="35"/>
-      <c r="E16" s="36"/>
-      <c r="F16" s="37"/>
-      <c r="G16" s="42"/>
-      <c r="H16" s="42"/>
-      <c r="I16" s="38"/>
+      <c r="C16" s="29"/>
+      <c r="D16" s="29"/>
+      <c r="E16" s="21"/>
+      <c r="F16" s="30"/>
+      <c r="G16" s="34"/>
+      <c r="H16" s="34"/>
+      <c r="I16" s="31"/>
     </row>
     <row r="17" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C17" s="35"/>
-      <c r="D17" s="35"/>
-      <c r="E17" s="36"/>
-      <c r="F17" s="37"/>
-      <c r="G17" s="42"/>
-      <c r="H17" s="42"/>
-      <c r="I17" s="38"/>
+      <c r="C17" s="29"/>
+      <c r="D17" s="29"/>
+      <c r="E17" s="21"/>
+      <c r="F17" s="30"/>
+      <c r="G17" s="34"/>
+      <c r="H17" s="34"/>
+      <c r="I17" s="31"/>
     </row>
     <row r="18" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C18" s="35"/>
-      <c r="D18" s="35"/>
-      <c r="E18" s="36"/>
-      <c r="F18" s="37"/>
-      <c r="G18" s="42"/>
-      <c r="H18" s="42"/>
-      <c r="I18" s="38"/>
+      <c r="C18" s="29"/>
+      <c r="D18" s="29"/>
+      <c r="E18" s="21"/>
+      <c r="F18" s="30"/>
+      <c r="G18" s="34"/>
+      <c r="H18" s="34"/>
+      <c r="I18" s="31"/>
     </row>
     <row r="19" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C19" s="35"/>
-      <c r="D19" s="35"/>
-      <c r="E19" s="36"/>
-      <c r="F19" s="37"/>
-      <c r="G19" s="42"/>
-      <c r="H19" s="42"/>
-      <c r="I19" s="38"/>
+      <c r="C19" s="29"/>
+      <c r="D19" s="29"/>
+      <c r="E19" s="21"/>
+      <c r="F19" s="30"/>
+      <c r="G19" s="34"/>
+      <c r="H19" s="34"/>
+      <c r="I19" s="31"/>
     </row>
     <row r="20" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C20" s="35"/>
-      <c r="D20" s="35"/>
-      <c r="E20" s="36"/>
-      <c r="F20" s="37"/>
-      <c r="G20" s="42"/>
-      <c r="H20" s="42"/>
-      <c r="I20" s="38"/>
+      <c r="C20" s="29"/>
+      <c r="D20" s="29"/>
+      <c r="E20" s="21"/>
+      <c r="F20" s="30"/>
+      <c r="G20" s="34"/>
+      <c r="H20" s="34"/>
+      <c r="I20" s="31"/>
     </row>
     <row r="21" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C21" s="35"/>
-      <c r="D21" s="35"/>
-      <c r="E21" s="36"/>
-      <c r="F21" s="37"/>
-      <c r="G21" s="42"/>
-      <c r="H21" s="42"/>
-      <c r="I21" s="38"/>
+      <c r="C21" s="29"/>
+      <c r="D21" s="29"/>
+      <c r="E21" s="21"/>
+      <c r="F21" s="30"/>
+      <c r="G21" s="34"/>
+      <c r="H21" s="34"/>
+      <c r="I21" s="31"/>
     </row>
     <row r="22" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C22" s="35"/>
-      <c r="D22" s="35"/>
-      <c r="E22" s="36"/>
-      <c r="F22" s="37"/>
-      <c r="G22" s="42"/>
-      <c r="H22" s="42"/>
-      <c r="I22" s="38"/>
+      <c r="C22" s="29"/>
+      <c r="D22" s="29"/>
+      <c r="E22" s="21"/>
+      <c r="F22" s="30"/>
+      <c r="G22" s="34"/>
+      <c r="H22" s="34"/>
+      <c r="I22" s="31"/>
     </row>
     <row r="23" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C23" s="35"/>
-      <c r="D23" s="35"/>
-      <c r="E23" s="36"/>
-      <c r="F23" s="37"/>
-      <c r="G23" s="42"/>
-      <c r="H23" s="42"/>
-      <c r="I23" s="38"/>
+      <c r="C23" s="29"/>
+      <c r="D23" s="29"/>
+      <c r="E23" s="21"/>
+      <c r="F23" s="30"/>
+      <c r="G23" s="34"/>
+      <c r="H23" s="34"/>
+      <c r="I23" s="31"/>
     </row>
     <row r="24" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C24" s="35"/>
-      <c r="D24" s="35"/>
-      <c r="E24" s="36"/>
-      <c r="F24" s="37"/>
-      <c r="G24" s="42"/>
-      <c r="H24" s="42"/>
-      <c r="I24" s="38"/>
+      <c r="C24" s="29"/>
+      <c r="D24" s="29"/>
+      <c r="E24" s="21"/>
+      <c r="F24" s="30"/>
+      <c r="G24" s="34"/>
+      <c r="H24" s="34"/>
+      <c r="I24" s="31"/>
     </row>
     <row r="25" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C25" s="35"/>
-      <c r="D25" s="35"/>
-      <c r="E25" s="36"/>
-      <c r="F25" s="37"/>
-      <c r="G25" s="42"/>
-      <c r="H25" s="42"/>
-      <c r="I25" s="38"/>
+      <c r="C25" s="29"/>
+      <c r="D25" s="29"/>
+      <c r="E25" s="21"/>
+      <c r="F25" s="30"/>
+      <c r="G25" s="34"/>
+      <c r="H25" s="34"/>
+      <c r="I25" s="31"/>
     </row>
     <row r="26" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C26" s="35"/>
-      <c r="D26" s="35"/>
-      <c r="E26" s="36"/>
-      <c r="F26" s="37"/>
-      <c r="G26" s="42"/>
-      <c r="H26" s="42"/>
-      <c r="I26" s="38"/>
+      <c r="C26" s="29"/>
+      <c r="D26" s="29"/>
+      <c r="E26" s="21"/>
+      <c r="F26" s="30"/>
+      <c r="G26" s="34"/>
+      <c r="H26" s="34"/>
+      <c r="I26" s="31"/>
     </row>
     <row r="27" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C27" s="35"/>
-      <c r="D27" s="35"/>
-      <c r="E27" s="36"/>
-      <c r="F27" s="37"/>
-      <c r="G27" s="42"/>
-      <c r="H27" s="42"/>
-      <c r="I27" s="38"/>
+      <c r="C27" s="29"/>
+      <c r="D27" s="29"/>
+      <c r="E27" s="21"/>
+      <c r="F27" s="30"/>
+      <c r="G27" s="34"/>
+      <c r="H27" s="34"/>
+      <c r="I27" s="31"/>
     </row>
     <row r="28" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C28" s="35"/>
-      <c r="D28" s="35"/>
-      <c r="E28" s="36"/>
-      <c r="F28" s="37"/>
-      <c r="G28" s="42"/>
-      <c r="H28" s="42"/>
-      <c r="I28" s="38"/>
+      <c r="C28" s="29"/>
+      <c r="D28" s="29"/>
+      <c r="E28" s="21"/>
+      <c r="F28" s="30"/>
+      <c r="G28" s="34"/>
+      <c r="H28" s="34"/>
+      <c r="I28" s="31"/>
     </row>
     <row r="29" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C29" s="35"/>
-      <c r="D29" s="35"/>
-      <c r="E29" s="36"/>
-      <c r="F29" s="37"/>
-      <c r="G29" s="42"/>
-      <c r="H29" s="42"/>
-      <c r="I29" s="38"/>
+      <c r="C29" s="29"/>
+      <c r="D29" s="29"/>
+      <c r="E29" s="21"/>
+      <c r="F29" s="30"/>
+      <c r="G29" s="34"/>
+      <c r="H29" s="34"/>
+      <c r="I29" s="31"/>
     </row>
     <row r="30" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C30" s="35"/>
-      <c r="D30" s="35"/>
-      <c r="E30" s="36"/>
-      <c r="F30" s="37"/>
-      <c r="G30" s="42"/>
-      <c r="H30" s="42"/>
-      <c r="I30" s="38"/>
+      <c r="C30" s="29"/>
+      <c r="D30" s="29"/>
+      <c r="E30" s="21"/>
+      <c r="F30" s="30"/>
+      <c r="G30" s="34"/>
+      <c r="H30" s="34"/>
+      <c r="I30" s="31"/>
     </row>
     <row r="31" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C31" s="35"/>
-      <c r="D31" s="35"/>
-      <c r="E31" s="36"/>
-      <c r="F31" s="37"/>
-      <c r="G31" s="42"/>
-      <c r="H31" s="42"/>
-      <c r="I31" s="38"/>
+      <c r="C31" s="29"/>
+      <c r="D31" s="29"/>
+      <c r="E31" s="21"/>
+      <c r="F31" s="30"/>
+      <c r="G31" s="34"/>
+      <c r="H31" s="34"/>
+      <c r="I31" s="31"/>
     </row>
     <row r="32" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C32" s="35"/>
-      <c r="D32" s="35"/>
-      <c r="E32" s="36"/>
-      <c r="F32" s="37"/>
-      <c r="G32" s="42"/>
-      <c r="H32" s="42"/>
-      <c r="I32" s="38"/>
+      <c r="C32" s="29"/>
+      <c r="D32" s="29"/>
+      <c r="E32" s="21"/>
+      <c r="F32" s="30"/>
+      <c r="G32" s="34"/>
+      <c r="H32" s="34"/>
+      <c r="I32" s="31"/>
     </row>
     <row r="33" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C33" s="35"/>
-      <c r="D33" s="35"/>
-      <c r="E33" s="36"/>
-      <c r="F33" s="37"/>
-      <c r="G33" s="42"/>
-      <c r="H33" s="42"/>
-      <c r="I33" s="38"/>
+      <c r="C33" s="29"/>
+      <c r="D33" s="29"/>
+      <c r="E33" s="21"/>
+      <c r="F33" s="30"/>
+      <c r="G33" s="34"/>
+      <c r="H33" s="34"/>
+      <c r="I33" s="31"/>
     </row>
     <row r="34" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C34" s="35"/>
-      <c r="D34" s="35"/>
-      <c r="E34" s="36"/>
-      <c r="F34" s="37"/>
-      <c r="G34" s="42"/>
-      <c r="H34" s="42"/>
-      <c r="I34" s="38"/>
+      <c r="C34" s="29"/>
+      <c r="D34" s="29"/>
+      <c r="E34" s="21"/>
+      <c r="F34" s="30"/>
+      <c r="G34" s="34"/>
+      <c r="H34" s="34"/>
+      <c r="I34" s="31"/>
     </row>
     <row r="35" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C35" s="35"/>
-      <c r="D35" s="35"/>
-      <c r="E35" s="36"/>
-      <c r="F35" s="37"/>
-      <c r="G35" s="42"/>
-      <c r="H35" s="42"/>
-      <c r="I35" s="38"/>
+      <c r="C35" s="29"/>
+      <c r="D35" s="29"/>
+      <c r="E35" s="21"/>
+      <c r="F35" s="30"/>
+      <c r="G35" s="34"/>
+      <c r="H35" s="34"/>
+      <c r="I35" s="31"/>
     </row>
     <row r="36" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C36" s="35"/>
-      <c r="D36" s="35"/>
-      <c r="E36" s="36"/>
-      <c r="F36" s="37"/>
-      <c r="G36" s="42"/>
-      <c r="H36" s="42"/>
-      <c r="I36" s="38"/>
+      <c r="C36" s="29"/>
+      <c r="D36" s="29"/>
+      <c r="E36" s="21"/>
+      <c r="F36" s="30"/>
+      <c r="G36" s="34"/>
+      <c r="H36" s="34"/>
+      <c r="I36" s="31"/>
     </row>
     <row r="37" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C37" s="35"/>
-      <c r="D37" s="35"/>
-      <c r="E37" s="36"/>
-      <c r="F37" s="37"/>
-      <c r="G37" s="42"/>
-      <c r="H37" s="42"/>
-      <c r="I37" s="38"/>
+      <c r="C37" s="29"/>
+      <c r="D37" s="29"/>
+      <c r="E37" s="21"/>
+      <c r="F37" s="30"/>
+      <c r="G37" s="34"/>
+      <c r="H37" s="34"/>
+      <c r="I37" s="31"/>
     </row>
     <row r="38" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C38" s="35"/>
-      <c r="D38" s="35"/>
-      <c r="E38" s="36"/>
-      <c r="F38" s="37"/>
-      <c r="G38" s="42"/>
-      <c r="H38" s="42"/>
-      <c r="I38" s="38"/>
+      <c r="C38" s="29"/>
+      <c r="D38" s="29"/>
+      <c r="E38" s="21"/>
+      <c r="F38" s="30"/>
+      <c r="G38" s="34"/>
+      <c r="H38" s="34"/>
+      <c r="I38" s="31"/>
     </row>
     <row r="39" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C39" s="35"/>
-      <c r="D39" s="35"/>
-      <c r="E39" s="36"/>
-      <c r="F39" s="37"/>
-      <c r="G39" s="42"/>
-      <c r="H39" s="42"/>
-      <c r="I39" s="38"/>
+      <c r="C39" s="29"/>
+      <c r="D39" s="29"/>
+      <c r="E39" s="21"/>
+      <c r="F39" s="30"/>
+      <c r="G39" s="34"/>
+      <c r="H39" s="34"/>
+      <c r="I39" s="31"/>
     </row>
     <row r="40" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C40" s="35"/>
-      <c r="D40" s="35"/>
-      <c r="E40" s="36"/>
-      <c r="F40" s="37"/>
-      <c r="G40" s="42"/>
-      <c r="H40" s="42"/>
-      <c r="I40" s="38"/>
+      <c r="C40" s="29"/>
+      <c r="D40" s="29"/>
+      <c r="E40" s="21"/>
+      <c r="F40" s="30"/>
+      <c r="G40" s="34"/>
+      <c r="H40" s="34"/>
+      <c r="I40" s="31"/>
     </row>
     <row r="41" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C41" s="35"/>
-      <c r="D41" s="35"/>
-      <c r="E41" s="36"/>
-      <c r="F41" s="37"/>
-      <c r="G41" s="42"/>
-      <c r="H41" s="42"/>
-      <c r="I41" s="38"/>
+      <c r="C41" s="29"/>
+      <c r="D41" s="29"/>
+      <c r="E41" s="21"/>
+      <c r="F41" s="30"/>
+      <c r="G41" s="34"/>
+      <c r="H41" s="34"/>
+      <c r="I41" s="31"/>
     </row>
     <row r="42" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C42" s="35"/>
-      <c r="D42" s="35"/>
-      <c r="E42" s="36"/>
-      <c r="F42" s="37"/>
-      <c r="G42" s="42"/>
-      <c r="H42" s="42"/>
-      <c r="I42" s="38"/>
+      <c r="C42" s="29"/>
+      <c r="D42" s="29"/>
+      <c r="E42" s="21"/>
+      <c r="F42" s="30"/>
+      <c r="G42" s="34"/>
+      <c r="H42" s="34"/>
+      <c r="I42" s="31"/>
     </row>
     <row r="43" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C43" s="35"/>
-      <c r="D43" s="35"/>
-      <c r="E43" s="36"/>
-      <c r="F43" s="37"/>
-      <c r="G43" s="42"/>
-      <c r="H43" s="42"/>
-      <c r="I43" s="38"/>
+      <c r="C43" s="29"/>
+      <c r="D43" s="29"/>
+      <c r="E43" s="21"/>
+      <c r="F43" s="30"/>
+      <c r="G43" s="34"/>
+      <c r="H43" s="34"/>
+      <c r="I43" s="31"/>
     </row>
     <row r="44" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C44" s="35"/>
-      <c r="D44" s="35"/>
-      <c r="E44" s="36"/>
-      <c r="F44" s="37"/>
-      <c r="G44" s="42"/>
-      <c r="H44" s="42"/>
-      <c r="I44" s="38"/>
+      <c r="C44" s="29"/>
+      <c r="D44" s="29"/>
+      <c r="E44" s="21"/>
+      <c r="F44" s="30"/>
+      <c r="G44" s="34"/>
+      <c r="H44" s="34"/>
+      <c r="I44" s="31"/>
     </row>
     <row r="45" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C45" s="35"/>
-      <c r="D45" s="35"/>
-      <c r="E45" s="36"/>
-      <c r="F45" s="37"/>
-      <c r="G45" s="42"/>
-      <c r="H45" s="42"/>
-      <c r="I45" s="38"/>
+      <c r="C45" s="29"/>
+      <c r="D45" s="29"/>
+      <c r="E45" s="21"/>
+      <c r="F45" s="30"/>
+      <c r="G45" s="34"/>
+      <c r="H45" s="34"/>
+      <c r="I45" s="31"/>
     </row>
     <row r="46" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C46" s="35"/>
-      <c r="D46" s="35"/>
-      <c r="E46" s="36"/>
-      <c r="F46" s="37"/>
-      <c r="G46" s="42"/>
-      <c r="H46" s="42"/>
-      <c r="I46" s="38"/>
+      <c r="C46" s="29"/>
+      <c r="D46" s="29"/>
+      <c r="E46" s="21"/>
+      <c r="F46" s="30"/>
+      <c r="G46" s="34"/>
+      <c r="H46" s="34"/>
+      <c r="I46" s="31"/>
     </row>
     <row r="47" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C47" s="35"/>
-      <c r="D47" s="35"/>
-      <c r="E47" s="36"/>
-      <c r="F47" s="37"/>
-      <c r="G47" s="42"/>
-      <c r="H47" s="42"/>
-      <c r="I47" s="38"/>
+      <c r="C47" s="29"/>
+      <c r="D47" s="29"/>
+      <c r="E47" s="21"/>
+      <c r="F47" s="30"/>
+      <c r="G47" s="34"/>
+      <c r="H47" s="34"/>
+      <c r="I47" s="31"/>
     </row>
     <row r="48" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C48" s="35"/>
-      <c r="D48" s="35"/>
-      <c r="E48" s="36"/>
-      <c r="F48" s="37"/>
-      <c r="G48" s="42"/>
-      <c r="H48" s="42"/>
-      <c r="I48" s="38"/>
+      <c r="C48" s="29"/>
+      <c r="D48" s="29"/>
+      <c r="E48" s="21"/>
+      <c r="F48" s="30"/>
+      <c r="G48" s="34"/>
+      <c r="H48" s="34"/>
+      <c r="I48" s="31"/>
     </row>
     <row r="49" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C49" s="35"/>
-      <c r="D49" s="35"/>
-      <c r="E49" s="36"/>
-      <c r="F49" s="37"/>
-      <c r="G49" s="42"/>
-      <c r="H49" s="42"/>
-      <c r="I49" s="38"/>
+      <c r="C49" s="29"/>
+      <c r="D49" s="29"/>
+      <c r="E49" s="21"/>
+      <c r="F49" s="30"/>
+      <c r="G49" s="34"/>
+      <c r="H49" s="34"/>
+      <c r="I49" s="31"/>
     </row>
     <row r="50" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C50" s="35"/>
-      <c r="D50" s="35"/>
-      <c r="E50" s="36"/>
-      <c r="F50" s="37"/>
-      <c r="G50" s="42"/>
-      <c r="H50" s="42"/>
-      <c r="I50" s="38"/>
+      <c r="C50" s="29"/>
+      <c r="D50" s="29"/>
+      <c r="E50" s="21"/>
+      <c r="F50" s="30"/>
+      <c r="G50" s="34"/>
+      <c r="H50" s="34"/>
+      <c r="I50" s="31"/>
     </row>
     <row r="51" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C51" s="35"/>
-      <c r="D51" s="35"/>
-      <c r="E51" s="36"/>
-      <c r="F51" s="37"/>
-      <c r="G51" s="42"/>
-      <c r="H51" s="42"/>
-      <c r="I51" s="38"/>
+      <c r="C51" s="29"/>
+      <c r="D51" s="29"/>
+      <c r="E51" s="21"/>
+      <c r="F51" s="30"/>
+      <c r="G51" s="34"/>
+      <c r="H51" s="34"/>
+      <c r="I51" s="31"/>
     </row>
     <row r="52" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C52" s="35"/>
-      <c r="D52" s="35"/>
-      <c r="E52" s="36"/>
-      <c r="F52" s="37"/>
-      <c r="G52" s="42"/>
-      <c r="H52" s="42"/>
-      <c r="I52" s="38"/>
+      <c r="C52" s="29"/>
+      <c r="D52" s="29"/>
+      <c r="E52" s="21"/>
+      <c r="F52" s="30"/>
+      <c r="G52" s="34"/>
+      <c r="H52" s="34"/>
+      <c r="I52" s="31"/>
     </row>
     <row r="53" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C53" s="35"/>
-      <c r="D53" s="35"/>
-      <c r="E53" s="36"/>
-      <c r="F53" s="37"/>
-      <c r="G53" s="42"/>
-      <c r="H53" s="42"/>
-      <c r="I53" s="38"/>
+      <c r="C53" s="29"/>
+      <c r="D53" s="29"/>
+      <c r="E53" s="21"/>
+      <c r="F53" s="30"/>
+      <c r="G53" s="34"/>
+      <c r="H53" s="34"/>
+      <c r="I53" s="31"/>
     </row>
     <row r="54" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C54" s="35"/>
-      <c r="D54" s="35"/>
-      <c r="E54" s="36"/>
-      <c r="F54" s="37"/>
-      <c r="G54" s="42"/>
-      <c r="H54" s="42"/>
-      <c r="I54" s="38"/>
+      <c r="C54" s="29"/>
+      <c r="D54" s="29"/>
+      <c r="E54" s="21"/>
+      <c r="F54" s="30"/>
+      <c r="G54" s="34"/>
+      <c r="H54" s="34"/>
+      <c r="I54" s="31"/>
     </row>
     <row r="55" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C55" s="35"/>
-      <c r="D55" s="35"/>
-      <c r="E55" s="36"/>
-      <c r="F55" s="37"/>
-      <c r="G55" s="42"/>
-      <c r="H55" s="42"/>
-      <c r="I55" s="38"/>
+      <c r="C55" s="29"/>
+      <c r="D55" s="29"/>
+      <c r="E55" s="21"/>
+      <c r="F55" s="30"/>
+      <c r="G55" s="34"/>
+      <c r="H55" s="34"/>
+      <c r="I55" s="31"/>
     </row>
     <row r="56" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C56" s="35"/>
-      <c r="D56" s="35"/>
-      <c r="E56" s="36"/>
-      <c r="F56" s="37"/>
-      <c r="G56" s="42"/>
-      <c r="H56" s="42"/>
-      <c r="I56" s="38"/>
+      <c r="C56" s="29"/>
+      <c r="D56" s="29"/>
+      <c r="E56" s="21"/>
+      <c r="F56" s="30"/>
+      <c r="G56" s="34"/>
+      <c r="H56" s="34"/>
+      <c r="I56" s="31"/>
     </row>
     <row r="57" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C57" s="35"/>
-      <c r="D57" s="35"/>
-      <c r="E57" s="36"/>
-      <c r="F57" s="37"/>
-      <c r="G57" s="42"/>
-      <c r="H57" s="42"/>
-      <c r="I57" s="38"/>
+      <c r="C57" s="29"/>
+      <c r="D57" s="29"/>
+      <c r="E57" s="21"/>
+      <c r="F57" s="30"/>
+      <c r="G57" s="34"/>
+      <c r="H57" s="34"/>
+      <c r="I57" s="31"/>
     </row>
     <row r="58" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C58" s="35"/>
-      <c r="D58" s="35"/>
-      <c r="E58" s="36"/>
-      <c r="F58" s="37"/>
-      <c r="G58" s="42"/>
-      <c r="H58" s="42"/>
-      <c r="I58" s="38"/>
+      <c r="C58" s="29"/>
+      <c r="D58" s="29"/>
+      <c r="E58" s="21"/>
+      <c r="F58" s="30"/>
+      <c r="G58" s="34"/>
+      <c r="H58" s="34"/>
+      <c r="I58" s="31"/>
     </row>
     <row r="59" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C59" s="35"/>
-      <c r="D59" s="35"/>
-      <c r="E59" s="36"/>
-      <c r="F59" s="37"/>
-      <c r="G59" s="42"/>
-      <c r="H59" s="42"/>
-      <c r="I59" s="38"/>
+      <c r="C59" s="29"/>
+      <c r="D59" s="29"/>
+      <c r="E59" s="21"/>
+      <c r="F59" s="30"/>
+      <c r="G59" s="34"/>
+      <c r="H59" s="34"/>
+      <c r="I59" s="31"/>
     </row>
     <row r="60" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C60" s="35"/>
-      <c r="D60" s="35"/>
-      <c r="E60" s="36"/>
-      <c r="F60" s="37"/>
-      <c r="G60" s="42"/>
-      <c r="H60" s="42"/>
-      <c r="I60" s="38"/>
+      <c r="C60" s="29"/>
+      <c r="D60" s="29"/>
+      <c r="E60" s="21"/>
+      <c r="F60" s="30"/>
+      <c r="G60" s="34"/>
+      <c r="H60" s="34"/>
+      <c r="I60" s="31"/>
     </row>
     <row r="61" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C61" s="35"/>
-      <c r="D61" s="35"/>
-      <c r="E61" s="36"/>
-      <c r="F61" s="37"/>
-      <c r="G61" s="42"/>
-      <c r="H61" s="42"/>
-      <c r="I61" s="38"/>
+      <c r="C61" s="29"/>
+      <c r="D61" s="29"/>
+      <c r="E61" s="21"/>
+      <c r="F61" s="30"/>
+      <c r="G61" s="34"/>
+      <c r="H61" s="34"/>
+      <c r="I61" s="31"/>
     </row>
     <row r="62" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C62" s="35"/>
-      <c r="D62" s="35"/>
-      <c r="E62" s="36"/>
-      <c r="F62" s="37"/>
-      <c r="G62" s="42"/>
-      <c r="H62" s="42"/>
-      <c r="I62" s="38"/>
+      <c r="C62" s="29"/>
+      <c r="D62" s="29"/>
+      <c r="E62" s="21"/>
+      <c r="F62" s="30"/>
+      <c r="G62" s="34"/>
+      <c r="H62" s="34"/>
+      <c r="I62" s="31"/>
     </row>
     <row r="63" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C63" s="35"/>
-      <c r="D63" s="35"/>
-      <c r="E63" s="36"/>
-      <c r="F63" s="37"/>
-      <c r="G63" s="42"/>
-      <c r="H63" s="42"/>
-      <c r="I63" s="38"/>
+      <c r="C63" s="29"/>
+      <c r="D63" s="29"/>
+      <c r="E63" s="21"/>
+      <c r="F63" s="30"/>
+      <c r="G63" s="34"/>
+      <c r="H63" s="34"/>
+      <c r="I63" s="31"/>
     </row>
     <row r="64" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C64" s="35"/>
-      <c r="D64" s="35"/>
-      <c r="E64" s="36"/>
-      <c r="F64" s="37"/>
-      <c r="G64" s="42"/>
-      <c r="H64" s="42"/>
-      <c r="I64" s="38"/>
+      <c r="C64" s="29"/>
+      <c r="D64" s="29"/>
+      <c r="E64" s="21"/>
+      <c r="F64" s="30"/>
+      <c r="G64" s="34"/>
+      <c r="H64" s="34"/>
+      <c r="I64" s="31"/>
     </row>
     <row r="65" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C65" s="35"/>
-      <c r="D65" s="35"/>
-      <c r="E65" s="36"/>
-      <c r="F65" s="37"/>
-      <c r="G65" s="42"/>
-      <c r="H65" s="42"/>
-      <c r="I65" s="38"/>
+      <c r="C65" s="29"/>
+      <c r="D65" s="29"/>
+      <c r="E65" s="21"/>
+      <c r="F65" s="30"/>
+      <c r="G65" s="34"/>
+      <c r="H65" s="34"/>
+      <c r="I65" s="31"/>
     </row>
     <row r="66" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C66" s="35"/>
-      <c r="D66" s="35"/>
-      <c r="E66" s="36"/>
-      <c r="F66" s="37"/>
-      <c r="G66" s="42"/>
-      <c r="H66" s="42"/>
-      <c r="I66" s="38"/>
+      <c r="C66" s="29"/>
+      <c r="D66" s="29"/>
+      <c r="E66" s="21"/>
+      <c r="F66" s="30"/>
+      <c r="G66" s="34"/>
+      <c r="H66" s="34"/>
+      <c r="I66" s="31"/>
     </row>
     <row r="67" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C67" s="35"/>
-      <c r="D67" s="35"/>
-      <c r="E67" s="36"/>
-      <c r="F67" s="37"/>
-      <c r="G67" s="42"/>
-      <c r="H67" s="42"/>
-      <c r="I67" s="38"/>
+      <c r="C67" s="29"/>
+      <c r="D67" s="29"/>
+      <c r="E67" s="21"/>
+      <c r="F67" s="30"/>
+      <c r="G67" s="34"/>
+      <c r="H67" s="34"/>
+      <c r="I67" s="31"/>
     </row>
     <row r="68" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C68" s="35"/>
-      <c r="D68" s="35"/>
-      <c r="E68" s="36"/>
-      <c r="F68" s="37"/>
-      <c r="G68" s="42"/>
-      <c r="H68" s="42"/>
-      <c r="I68" s="38"/>
+      <c r="C68" s="29"/>
+      <c r="D68" s="29"/>
+      <c r="E68" s="21"/>
+      <c r="F68" s="30"/>
+      <c r="G68" s="34"/>
+      <c r="H68" s="34"/>
+      <c r="I68" s="31"/>
     </row>
     <row r="69" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C69" s="35"/>
-      <c r="D69" s="35"/>
-      <c r="E69" s="36"/>
-      <c r="F69" s="37"/>
-      <c r="G69" s="42"/>
-      <c r="H69" s="42"/>
-      <c r="I69" s="38"/>
+      <c r="C69" s="29"/>
+      <c r="D69" s="29"/>
+      <c r="E69" s="21"/>
+      <c r="F69" s="30"/>
+      <c r="G69" s="34"/>
+      <c r="H69" s="34"/>
+      <c r="I69" s="31"/>
     </row>
     <row r="70" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C70" s="35"/>
-      <c r="D70" s="35"/>
-      <c r="E70" s="36"/>
-      <c r="F70" s="37"/>
-      <c r="G70" s="42"/>
-      <c r="H70" s="42"/>
-      <c r="I70" s="38"/>
+      <c r="C70" s="29"/>
+      <c r="D70" s="29"/>
+      <c r="E70" s="21"/>
+      <c r="F70" s="30"/>
+      <c r="G70" s="34"/>
+      <c r="H70" s="34"/>
+      <c r="I70" s="31"/>
     </row>
     <row r="71" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C71" s="35"/>
-      <c r="D71" s="35"/>
-      <c r="E71" s="36"/>
-      <c r="F71" s="37"/>
-      <c r="G71" s="42"/>
-      <c r="H71" s="42"/>
-      <c r="I71" s="38"/>
+      <c r="C71" s="29"/>
+      <c r="D71" s="29"/>
+      <c r="E71" s="21"/>
+      <c r="F71" s="30"/>
+      <c r="G71" s="34"/>
+      <c r="H71" s="34"/>
+      <c r="I71" s="31"/>
     </row>
     <row r="72" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C72" s="35"/>
-      <c r="D72" s="35"/>
-      <c r="E72" s="36"/>
-      <c r="F72" s="37"/>
-      <c r="G72" s="42"/>
-      <c r="H72" s="42"/>
-      <c r="I72" s="38"/>
+      <c r="C72" s="29"/>
+      <c r="D72" s="29"/>
+      <c r="E72" s="21"/>
+      <c r="F72" s="30"/>
+      <c r="G72" s="34"/>
+      <c r="H72" s="34"/>
+      <c r="I72" s="31"/>
     </row>
     <row r="73" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C73" s="35"/>
-      <c r="D73" s="35"/>
-      <c r="E73" s="36"/>
-      <c r="F73" s="37"/>
-      <c r="G73" s="42"/>
-      <c r="H73" s="42"/>
-      <c r="I73" s="38"/>
+      <c r="C73" s="29"/>
+      <c r="D73" s="29"/>
+      <c r="E73" s="21"/>
+      <c r="F73" s="30"/>
+      <c r="G73" s="34"/>
+      <c r="H73" s="34"/>
+      <c r="I73" s="31"/>
     </row>
     <row r="74" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C74" s="35"/>
-      <c r="D74" s="35"/>
-      <c r="E74" s="36"/>
-      <c r="F74" s="37"/>
-      <c r="G74" s="42"/>
-      <c r="H74" s="42"/>
-      <c r="I74" s="38"/>
+      <c r="C74" s="29"/>
+      <c r="D74" s="29"/>
+      <c r="E74" s="21"/>
+      <c r="F74" s="30"/>
+      <c r="G74" s="34"/>
+      <c r="H74" s="34"/>
+      <c r="I74" s="31"/>
     </row>
     <row r="75" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C75" s="35"/>
-      <c r="D75" s="35"/>
-      <c r="E75" s="36"/>
-      <c r="F75" s="37"/>
-      <c r="G75" s="42"/>
-      <c r="H75" s="42"/>
-      <c r="I75" s="38"/>
+      <c r="C75" s="29"/>
+      <c r="D75" s="29"/>
+      <c r="E75" s="21"/>
+      <c r="F75" s="30"/>
+      <c r="G75" s="34"/>
+      <c r="H75" s="34"/>
+      <c r="I75" s="31"/>
     </row>
     <row r="76" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C76" s="35"/>
-      <c r="D76" s="35"/>
-      <c r="E76" s="36"/>
-      <c r="F76" s="37"/>
-      <c r="G76" s="42"/>
-      <c r="H76" s="42"/>
-      <c r="I76" s="38"/>
+      <c r="C76" s="29"/>
+      <c r="D76" s="29"/>
+      <c r="E76" s="21"/>
+      <c r="F76" s="30"/>
+      <c r="G76" s="34"/>
+      <c r="H76" s="34"/>
+      <c r="I76" s="31"/>
     </row>
     <row r="77" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C77" s="35"/>
-      <c r="D77" s="35"/>
-      <c r="E77" s="36"/>
-      <c r="F77" s="37"/>
-      <c r="G77" s="42"/>
-      <c r="H77" s="42"/>
-      <c r="I77" s="38"/>
+      <c r="C77" s="29"/>
+      <c r="D77" s="29"/>
+      <c r="E77" s="21"/>
+      <c r="F77" s="30"/>
+      <c r="G77" s="34"/>
+      <c r="H77" s="34"/>
+      <c r="I77" s="31"/>
     </row>
     <row r="78" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C78" s="35"/>
-      <c r="D78" s="35"/>
-      <c r="E78" s="36"/>
-      <c r="F78" s="37"/>
-      <c r="G78" s="42"/>
-      <c r="H78" s="42"/>
-      <c r="I78" s="38"/>
+      <c r="C78" s="29"/>
+      <c r="D78" s="29"/>
+      <c r="E78" s="21"/>
+      <c r="F78" s="30"/>
+      <c r="G78" s="34"/>
+      <c r="H78" s="34"/>
+      <c r="I78" s="31"/>
     </row>
     <row r="79" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C79" s="35"/>
-      <c r="D79" s="35"/>
-      <c r="E79" s="36"/>
-      <c r="F79" s="37"/>
-      <c r="G79" s="42"/>
-      <c r="H79" s="42"/>
-      <c r="I79" s="38"/>
+      <c r="C79" s="29"/>
+      <c r="D79" s="29"/>
+      <c r="E79" s="21"/>
+      <c r="F79" s="30"/>
+      <c r="G79" s="34"/>
+      <c r="H79" s="34"/>
+      <c r="I79" s="31"/>
     </row>
     <row r="80" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C80" s="35"/>
-      <c r="D80" s="35"/>
-      <c r="E80" s="36"/>
-      <c r="F80" s="37"/>
-      <c r="G80" s="42"/>
-      <c r="H80" s="42"/>
-      <c r="I80" s="38"/>
+      <c r="C80" s="29"/>
+      <c r="D80" s="29"/>
+      <c r="E80" s="21"/>
+      <c r="F80" s="30"/>
+      <c r="G80" s="34"/>
+      <c r="H80" s="34"/>
+      <c r="I80" s="31"/>
     </row>
     <row r="81" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C81" s="35"/>
-      <c r="D81" s="35"/>
-      <c r="E81" s="36"/>
-      <c r="F81" s="37"/>
-      <c r="G81" s="42"/>
-      <c r="H81" s="42"/>
-      <c r="I81" s="38"/>
+      <c r="C81" s="29"/>
+      <c r="D81" s="29"/>
+      <c r="E81" s="21"/>
+      <c r="F81" s="30"/>
+      <c r="G81" s="34"/>
+      <c r="H81" s="34"/>
+      <c r="I81" s="31"/>
     </row>
     <row r="82" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C82" s="35"/>
-      <c r="D82" s="35"/>
-      <c r="E82" s="36"/>
-      <c r="F82" s="37"/>
-      <c r="G82" s="42"/>
-      <c r="H82" s="42"/>
-      <c r="I82" s="38"/>
+      <c r="C82" s="29"/>
+      <c r="D82" s="29"/>
+      <c r="E82" s="21"/>
+      <c r="F82" s="30"/>
+      <c r="G82" s="34"/>
+      <c r="H82" s="34"/>
+      <c r="I82" s="31"/>
     </row>
     <row r="83" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C83" s="35"/>
-      <c r="D83" s="35"/>
-      <c r="E83" s="36"/>
-      <c r="F83" s="37"/>
-      <c r="G83" s="42"/>
-      <c r="H83" s="42"/>
-      <c r="I83" s="38"/>
+      <c r="C83" s="29"/>
+      <c r="D83" s="29"/>
+      <c r="E83" s="21"/>
+      <c r="F83" s="30"/>
+      <c r="G83" s="34"/>
+      <c r="H83" s="34"/>
+      <c r="I83" s="31"/>
     </row>
     <row r="84" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C84" s="35"/>
-      <c r="D84" s="35"/>
-      <c r="E84" s="36"/>
-      <c r="F84" s="37"/>
-      <c r="G84" s="42"/>
-      <c r="H84" s="42"/>
-      <c r="I84" s="38"/>
+      <c r="C84" s="29"/>
+      <c r="D84" s="29"/>
+      <c r="E84" s="21"/>
+      <c r="F84" s="30"/>
+      <c r="G84" s="34"/>
+      <c r="H84" s="34"/>
+      <c r="I84" s="31"/>
     </row>
     <row r="85" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C85" s="35"/>
-      <c r="D85" s="35"/>
-      <c r="E85" s="36"/>
-      <c r="F85" s="37"/>
-      <c r="G85" s="42"/>
-      <c r="H85" s="42"/>
-      <c r="I85" s="38"/>
+      <c r="C85" s="29"/>
+      <c r="D85" s="29"/>
+      <c r="E85" s="21"/>
+      <c r="F85" s="30"/>
+      <c r="G85" s="34"/>
+      <c r="H85" s="34"/>
+      <c r="I85" s="31"/>
     </row>
     <row r="86" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C86" s="35"/>
-      <c r="D86" s="35"/>
-      <c r="E86" s="36"/>
-      <c r="F86" s="37"/>
-      <c r="G86" s="42"/>
-      <c r="H86" s="42"/>
-      <c r="I86" s="38"/>
+      <c r="C86" s="29"/>
+      <c r="D86" s="29"/>
+      <c r="E86" s="21"/>
+      <c r="F86" s="30"/>
+      <c r="G86" s="34"/>
+      <c r="H86" s="34"/>
+      <c r="I86" s="31"/>
     </row>
     <row r="87" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C87" s="35"/>
-      <c r="D87" s="35"/>
-      <c r="E87" s="36"/>
-      <c r="F87" s="37"/>
-      <c r="G87" s="42"/>
-      <c r="H87" s="42"/>
-      <c r="I87" s="38"/>
+      <c r="C87" s="29"/>
+      <c r="D87" s="29"/>
+      <c r="E87" s="21"/>
+      <c r="F87" s="30"/>
+      <c r="G87" s="34"/>
+      <c r="H87" s="34"/>
+      <c r="I87" s="31"/>
     </row>
     <row r="88" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C88" s="35"/>
-      <c r="D88" s="35"/>
-      <c r="E88" s="36"/>
-      <c r="F88" s="37"/>
-      <c r="G88" s="42"/>
-      <c r="H88" s="42"/>
-      <c r="I88" s="38"/>
+      <c r="C88" s="29"/>
+      <c r="D88" s="29"/>
+      <c r="E88" s="21"/>
+      <c r="F88" s="30"/>
+      <c r="G88" s="34"/>
+      <c r="H88" s="34"/>
+      <c r="I88" s="31"/>
     </row>
     <row r="89" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C89" s="35"/>
-      <c r="D89" s="35"/>
-      <c r="E89" s="36"/>
-      <c r="F89" s="37"/>
-      <c r="G89" s="42"/>
-      <c r="H89" s="42"/>
-      <c r="I89" s="38"/>
+      <c r="C89" s="29"/>
+      <c r="D89" s="29"/>
+      <c r="E89" s="21"/>
+      <c r="F89" s="30"/>
+      <c r="G89" s="34"/>
+      <c r="H89" s="34"/>
+      <c r="I89" s="31"/>
     </row>
     <row r="90" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C90" s="35"/>
-      <c r="D90" s="35"/>
-      <c r="E90" s="36"/>
-      <c r="F90" s="37"/>
-      <c r="G90" s="42"/>
-      <c r="H90" s="42"/>
-      <c r="I90" s="38"/>
+      <c r="C90" s="29"/>
+      <c r="D90" s="29"/>
+      <c r="E90" s="21"/>
+      <c r="F90" s="30"/>
+      <c r="G90" s="34"/>
+      <c r="H90" s="34"/>
+      <c r="I90" s="31"/>
     </row>
     <row r="91" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C91" s="35"/>
-      <c r="D91" s="35"/>
-      <c r="E91" s="36"/>
-      <c r="F91" s="37"/>
-      <c r="G91" s="42"/>
-      <c r="H91" s="42"/>
-      <c r="I91" s="38"/>
+      <c r="C91" s="29"/>
+      <c r="D91" s="29"/>
+      <c r="E91" s="21"/>
+      <c r="F91" s="30"/>
+      <c r="G91" s="34"/>
+      <c r="H91" s="34"/>
+      <c r="I91" s="31"/>
     </row>
     <row r="92" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C92" s="35"/>
-      <c r="D92" s="35"/>
-      <c r="E92" s="36"/>
-      <c r="F92" s="37"/>
-      <c r="G92" s="42"/>
-      <c r="H92" s="42"/>
-      <c r="I92" s="38"/>
+      <c r="C92" s="29"/>
+      <c r="D92" s="29"/>
+      <c r="E92" s="21"/>
+      <c r="F92" s="30"/>
+      <c r="G92" s="34"/>
+      <c r="H92" s="34"/>
+      <c r="I92" s="31"/>
     </row>
     <row r="93" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C93" s="35"/>
-      <c r="D93" s="35"/>
-      <c r="E93" s="36"/>
-      <c r="F93" s="37"/>
-      <c r="G93" s="42"/>
-      <c r="H93" s="42"/>
-      <c r="I93" s="38"/>
+      <c r="C93" s="29"/>
+      <c r="D93" s="29"/>
+      <c r="E93" s="21"/>
+      <c r="F93" s="30"/>
+      <c r="G93" s="34"/>
+      <c r="H93" s="34"/>
+      <c r="I93" s="31"/>
     </row>
     <row r="94" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C94" s="35"/>
-      <c r="D94" s="35"/>
-      <c r="E94" s="36"/>
-      <c r="F94" s="37"/>
-      <c r="G94" s="42"/>
-      <c r="H94" s="42"/>
-      <c r="I94" s="38"/>
+      <c r="C94" s="29"/>
+      <c r="D94" s="29"/>
+      <c r="E94" s="21"/>
+      <c r="F94" s="30"/>
+      <c r="G94" s="34"/>
+      <c r="H94" s="34"/>
+      <c r="I94" s="31"/>
     </row>
     <row r="95" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C95" s="35"/>
-      <c r="D95" s="35"/>
-      <c r="E95" s="36"/>
-      <c r="F95" s="37"/>
-      <c r="G95" s="42"/>
-      <c r="H95" s="42"/>
-      <c r="I95" s="38"/>
+      <c r="C95" s="29"/>
+      <c r="D95" s="29"/>
+      <c r="E95" s="21"/>
+      <c r="F95" s="30"/>
+      <c r="G95" s="34"/>
+      <c r="H95" s="34"/>
+      <c r="I95" s="31"/>
     </row>
     <row r="96" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C96" s="35"/>
-      <c r="D96" s="35"/>
-      <c r="E96" s="36"/>
-      <c r="F96" s="37"/>
-      <c r="G96" s="42"/>
-      <c r="H96" s="42"/>
-      <c r="I96" s="38"/>
+      <c r="C96" s="29"/>
+      <c r="D96" s="29"/>
+      <c r="E96" s="21"/>
+      <c r="F96" s="30"/>
+      <c r="G96" s="34"/>
+      <c r="H96" s="34"/>
+      <c r="I96" s="31"/>
     </row>
     <row r="97" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C97" s="35"/>
-      <c r="D97" s="35"/>
-      <c r="E97" s="36"/>
-      <c r="F97" s="37"/>
-      <c r="G97" s="42"/>
-      <c r="H97" s="42"/>
-      <c r="I97" s="38"/>
+      <c r="C97" s="29"/>
+      <c r="D97" s="29"/>
+      <c r="E97" s="21"/>
+      <c r="F97" s="30"/>
+      <c r="G97" s="34"/>
+      <c r="H97" s="34"/>
+      <c r="I97" s="31"/>
     </row>
     <row r="98" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C98" s="35"/>
-      <c r="D98" s="35"/>
-      <c r="E98" s="36"/>
-      <c r="F98" s="37"/>
-      <c r="G98" s="42"/>
-      <c r="H98" s="42"/>
-      <c r="I98" s="38"/>
+      <c r="C98" s="29"/>
+      <c r="D98" s="29"/>
+      <c r="E98" s="21"/>
+      <c r="F98" s="30"/>
+      <c r="G98" s="34"/>
+      <c r="H98" s="34"/>
+      <c r="I98" s="31"/>
     </row>
     <row r="99" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C99" s="35"/>
-      <c r="D99" s="35"/>
-      <c r="E99" s="36"/>
-      <c r="F99" s="37"/>
-      <c r="G99" s="42"/>
-      <c r="H99" s="42"/>
-      <c r="I99" s="38"/>
+      <c r="C99" s="29"/>
+      <c r="D99" s="29"/>
+      <c r="E99" s="21"/>
+      <c r="F99" s="30"/>
+      <c r="G99" s="34"/>
+      <c r="H99" s="34"/>
+      <c r="I99" s="31"/>
     </row>
     <row r="100" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C100" s="35"/>
-      <c r="D100" s="35"/>
-      <c r="E100" s="36"/>
-      <c r="F100" s="37"/>
-      <c r="G100" s="42"/>
-      <c r="H100" s="42"/>
-      <c r="I100" s="38"/>
+      <c r="C100" s="29"/>
+      <c r="D100" s="29"/>
+      <c r="E100" s="21"/>
+      <c r="F100" s="30"/>
+      <c r="G100" s="34"/>
+      <c r="H100" s="34"/>
+      <c r="I100" s="31"/>
     </row>
     <row r="101" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C101" s="35"/>
-      <c r="D101" s="35"/>
-      <c r="E101" s="36"/>
-      <c r="F101" s="37"/>
-      <c r="G101" s="42"/>
-      <c r="H101" s="42"/>
-      <c r="I101" s="38"/>
+      <c r="C101" s="29"/>
+      <c r="D101" s="29"/>
+      <c r="E101" s="21"/>
+      <c r="F101" s="30"/>
+      <c r="G101" s="34"/>
+      <c r="H101" s="34"/>
+      <c r="I101" s="31"/>
     </row>
     <row r="102" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C102" s="35"/>
-      <c r="D102" s="35"/>
-      <c r="E102" s="36"/>
-      <c r="F102" s="37"/>
-      <c r="G102" s="42"/>
-      <c r="H102" s="42"/>
-      <c r="I102" s="38"/>
+      <c r="C102" s="29"/>
+      <c r="D102" s="29"/>
+      <c r="E102" s="21"/>
+      <c r="F102" s="30"/>
+      <c r="G102" s="34"/>
+      <c r="H102" s="34"/>
+      <c r="I102" s="31"/>
     </row>
     <row r="103" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C103" s="35"/>
-      <c r="D103" s="35"/>
-      <c r="E103" s="36"/>
-      <c r="F103" s="37"/>
-      <c r="G103" s="42"/>
-      <c r="H103" s="42"/>
-      <c r="I103" s="38"/>
+      <c r="C103" s="29"/>
+      <c r="D103" s="29"/>
+      <c r="E103" s="21"/>
+      <c r="F103" s="30"/>
+      <c r="G103" s="34"/>
+      <c r="H103" s="34"/>
+      <c r="I103" s="31"/>
     </row>
     <row r="104" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C104" s="35"/>
-      <c r="D104" s="35"/>
-      <c r="E104" s="36"/>
-      <c r="F104" s="37"/>
-      <c r="G104" s="42"/>
-      <c r="H104" s="42"/>
-      <c r="I104" s="38"/>
+      <c r="C104" s="29"/>
+      <c r="D104" s="29"/>
+      <c r="E104" s="21"/>
+      <c r="F104" s="30"/>
+      <c r="G104" s="34"/>
+      <c r="H104" s="34"/>
+      <c r="I104" s="31"/>
     </row>
     <row r="105" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C105" s="35"/>
-      <c r="D105" s="35"/>
-      <c r="E105" s="36"/>
-      <c r="F105" s="37"/>
-      <c r="G105" s="42"/>
-      <c r="H105" s="42"/>
-      <c r="I105" s="38"/>
+      <c r="C105" s="29"/>
+      <c r="D105" s="29"/>
+      <c r="E105" s="21"/>
+      <c r="F105" s="30"/>
+      <c r="G105" s="34"/>
+      <c r="H105" s="34"/>
+      <c r="I105" s="31"/>
     </row>
     <row r="106" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C106" s="35"/>
-      <c r="D106" s="35"/>
-      <c r="E106" s="36"/>
-      <c r="F106" s="37"/>
-      <c r="G106" s="42"/>
-      <c r="H106" s="42"/>
-      <c r="I106" s="38"/>
+      <c r="C106" s="29"/>
+      <c r="D106" s="29"/>
+      <c r="E106" s="21"/>
+      <c r="F106" s="30"/>
+      <c r="G106" s="34"/>
+      <c r="H106" s="34"/>
+      <c r="I106" s="31"/>
     </row>
     <row r="107" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C107" s="35"/>
-      <c r="D107" s="35"/>
-      <c r="E107" s="36"/>
-      <c r="F107" s="37"/>
-      <c r="G107" s="42"/>
-      <c r="H107" s="42"/>
-      <c r="I107" s="38"/>
+      <c r="C107" s="29"/>
+      <c r="D107" s="29"/>
+      <c r="E107" s="21"/>
+      <c r="F107" s="30"/>
+      <c r="G107" s="34"/>
+      <c r="H107" s="34"/>
+      <c r="I107" s="31"/>
     </row>
     <row r="108" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C108" s="35"/>
-      <c r="D108" s="35"/>
-      <c r="E108" s="36"/>
-      <c r="F108" s="37"/>
-      <c r="G108" s="42"/>
-      <c r="H108" s="42"/>
-      <c r="I108" s="38"/>
+      <c r="C108" s="29"/>
+      <c r="D108" s="29"/>
+      <c r="E108" s="21"/>
+      <c r="F108" s="30"/>
+      <c r="G108" s="34"/>
+      <c r="H108" s="34"/>
+      <c r="I108" s="31"/>
     </row>
     <row r="109" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C109" s="35"/>
-      <c r="D109" s="35"/>
-      <c r="E109" s="36"/>
-      <c r="F109" s="37"/>
-      <c r="G109" s="42"/>
-      <c r="H109" s="42"/>
-      <c r="I109" s="38"/>
+      <c r="C109" s="29"/>
+      <c r="D109" s="29"/>
+      <c r="E109" s="21"/>
+      <c r="F109" s="30"/>
+      <c r="G109" s="34"/>
+      <c r="H109" s="34"/>
+      <c r="I109" s="31"/>
     </row>
     <row r="110" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C110" s="35"/>
-      <c r="D110" s="35"/>
-      <c r="E110" s="36"/>
-      <c r="F110" s="37"/>
-      <c r="G110" s="42"/>
-      <c r="H110" s="42"/>
-      <c r="I110" s="38"/>
+      <c r="C110" s="29"/>
+      <c r="D110" s="29"/>
+      <c r="E110" s="21"/>
+      <c r="F110" s="30"/>
+      <c r="G110" s="34"/>
+      <c r="H110" s="34"/>
+      <c r="I110" s="31"/>
     </row>
     <row r="111" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C111" s="35"/>
-      <c r="D111" s="35"/>
-      <c r="E111" s="36"/>
-      <c r="F111" s="37"/>
-      <c r="G111" s="42"/>
-      <c r="H111" s="42"/>
-      <c r="I111" s="38"/>
+      <c r="C111" s="29"/>
+      <c r="D111" s="29"/>
+      <c r="E111" s="21"/>
+      <c r="F111" s="30"/>
+      <c r="G111" s="34"/>
+      <c r="H111" s="34"/>
+      <c r="I111" s="31"/>
     </row>
     <row r="112" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C112" s="35"/>
-      <c r="D112" s="35"/>
-      <c r="E112" s="36"/>
-      <c r="F112" s="37"/>
-      <c r="G112" s="42"/>
-      <c r="H112" s="42"/>
-      <c r="I112" s="38"/>
+      <c r="C112" s="29"/>
+      <c r="D112" s="29"/>
+      <c r="E112" s="21"/>
+      <c r="F112" s="30"/>
+      <c r="G112" s="34"/>
+      <c r="H112" s="34"/>
+      <c r="I112" s="31"/>
     </row>
     <row r="113" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C113" s="35"/>
-      <c r="D113" s="35"/>
-      <c r="E113" s="36"/>
-      <c r="F113" s="37"/>
-      <c r="G113" s="42"/>
-      <c r="H113" s="42"/>
-      <c r="I113" s="38"/>
+      <c r="C113" s="29"/>
+      <c r="D113" s="29"/>
+      <c r="E113" s="21"/>
+      <c r="F113" s="30"/>
+      <c r="G113" s="34"/>
+      <c r="H113" s="34"/>
+      <c r="I113" s="31"/>
     </row>
     <row r="114" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C114" s="35"/>
-      <c r="D114" s="35"/>
-      <c r="E114" s="36"/>
-      <c r="F114" s="37"/>
-      <c r="G114" s="42"/>
-      <c r="H114" s="42"/>
-      <c r="I114" s="38"/>
+      <c r="C114" s="29"/>
+      <c r="D114" s="29"/>
+      <c r="E114" s="21"/>
+      <c r="F114" s="30"/>
+      <c r="G114" s="34"/>
+      <c r="H114" s="34"/>
+      <c r="I114" s="31"/>
     </row>
     <row r="115" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C115" s="35"/>
-      <c r="D115" s="35"/>
-      <c r="E115" s="36"/>
-      <c r="F115" s="37"/>
-      <c r="G115" s="42"/>
-      <c r="H115" s="42"/>
-      <c r="I115" s="38"/>
+      <c r="C115" s="29"/>
+      <c r="D115" s="29"/>
+      <c r="E115" s="21"/>
+      <c r="F115" s="30"/>
+      <c r="G115" s="34"/>
+      <c r="H115" s="34"/>
+      <c r="I115" s="31"/>
     </row>
     <row r="116" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C116" s="35"/>
-      <c r="D116" s="35"/>
-      <c r="E116" s="36"/>
-      <c r="F116" s="37"/>
-      <c r="G116" s="42"/>
-      <c r="H116" s="42"/>
-      <c r="I116" s="38"/>
+      <c r="C116" s="29"/>
+      <c r="D116" s="29"/>
+      <c r="E116" s="21"/>
+      <c r="F116" s="30"/>
+      <c r="G116" s="34"/>
+      <c r="H116" s="34"/>
+      <c r="I116" s="31"/>
     </row>
     <row r="117" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C117" s="35"/>
-      <c r="D117" s="35"/>
-      <c r="E117" s="36"/>
-      <c r="F117" s="37"/>
-      <c r="G117" s="42"/>
-      <c r="H117" s="42"/>
-      <c r="I117" s="38"/>
+      <c r="C117" s="29"/>
+      <c r="D117" s="29"/>
+      <c r="E117" s="21"/>
+      <c r="F117" s="30"/>
+      <c r="G117" s="34"/>
+      <c r="H117" s="34"/>
+      <c r="I117" s="31"/>
     </row>
     <row r="118" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C118" s="35"/>
-      <c r="D118" s="35"/>
-      <c r="E118" s="36"/>
-      <c r="F118" s="37"/>
-      <c r="G118" s="42"/>
-      <c r="H118" s="42"/>
-      <c r="I118" s="38"/>
+      <c r="C118" s="29"/>
+      <c r="D118" s="29"/>
+      <c r="E118" s="21"/>
+      <c r="F118" s="30"/>
+      <c r="G118" s="34"/>
+      <c r="H118" s="34"/>
+      <c r="I118" s="31"/>
     </row>
     <row r="119" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C119" s="35"/>
-      <c r="D119" s="35"/>
-      <c r="E119" s="36"/>
-      <c r="F119" s="37"/>
-      <c r="G119" s="42"/>
-      <c r="H119" s="42"/>
-      <c r="I119" s="38"/>
+      <c r="C119" s="29"/>
+      <c r="D119" s="29"/>
+      <c r="E119" s="21"/>
+      <c r="F119" s="30"/>
+      <c r="G119" s="34"/>
+      <c r="H119" s="34"/>
+      <c r="I119" s="31"/>
     </row>
     <row r="120" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C120" s="35"/>
-      <c r="D120" s="35"/>
-      <c r="E120" s="36"/>
-      <c r="F120" s="37"/>
-      <c r="G120" s="42"/>
-      <c r="H120" s="42"/>
-      <c r="I120" s="38"/>
+      <c r="C120" s="29"/>
+      <c r="D120" s="29"/>
+      <c r="E120" s="21"/>
+      <c r="F120" s="30"/>
+      <c r="G120" s="34"/>
+      <c r="H120" s="34"/>
+      <c r="I120" s="31"/>
     </row>
     <row r="121" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C121" s="35"/>
-      <c r="D121" s="35"/>
-      <c r="E121" s="36"/>
-      <c r="F121" s="37"/>
-      <c r="G121" s="42"/>
-      <c r="H121" s="42"/>
-      <c r="I121" s="38"/>
+      <c r="C121" s="29"/>
+      <c r="D121" s="29"/>
+      <c r="E121" s="21"/>
+      <c r="F121" s="30"/>
+      <c r="G121" s="34"/>
+      <c r="H121" s="34"/>
+      <c r="I121" s="31"/>
     </row>
     <row r="122" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C122" s="35"/>
-      <c r="D122" s="35"/>
-      <c r="E122" s="36"/>
-      <c r="F122" s="37"/>
-      <c r="G122" s="42"/>
-      <c r="H122" s="42"/>
-      <c r="I122" s="38"/>
+      <c r="C122" s="29"/>
+      <c r="D122" s="29"/>
+      <c r="E122" s="21"/>
+      <c r="F122" s="30"/>
+      <c r="G122" s="34"/>
+      <c r="H122" s="34"/>
+      <c r="I122" s="31"/>
     </row>
     <row r="123" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C123" s="35"/>
-      <c r="D123" s="35"/>
-      <c r="E123" s="36"/>
-      <c r="F123" s="37"/>
-      <c r="G123" s="42"/>
-      <c r="H123" s="42"/>
-      <c r="I123" s="38"/>
+      <c r="C123" s="29"/>
+      <c r="D123" s="29"/>
+      <c r="E123" s="21"/>
+      <c r="F123" s="30"/>
+      <c r="G123" s="34"/>
+      <c r="H123" s="34"/>
+      <c r="I123" s="31"/>
     </row>
     <row r="124" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C124" s="35"/>
-      <c r="D124" s="35"/>
-      <c r="E124" s="36"/>
-      <c r="F124" s="37"/>
-      <c r="G124" s="42"/>
-      <c r="H124" s="42"/>
-      <c r="I124" s="38"/>
+      <c r="C124" s="29"/>
+      <c r="D124" s="29"/>
+      <c r="E124" s="21"/>
+      <c r="F124" s="30"/>
+      <c r="G124" s="34"/>
+      <c r="H124" s="34"/>
+      <c r="I124" s="31"/>
     </row>
     <row r="125" spans="3:9" x14ac:dyDescent="0.35">
-      <c r="C125" s="35"/>
-      <c r="D125" s="35"/>
-      <c r="E125" s="36"/>
-      <c r="F125" s="37"/>
-      <c r="G125" s="42"/>
-      <c r="H125" s="42"/>
-      <c r="I125" s="38"/>
+      <c r="C125" s="29"/>
+      <c r="D125" s="29"/>
+      <c r="E125" s="21"/>
+      <c r="F125" s="30"/>
+      <c r="G125" s="34"/>
+      <c r="H125" s="34"/>
+      <c r="I125" s="31"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2901,7 +2892,7 @@
     <col min="9" max="9" width="32.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:9" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="15" t="s">
         <v>66</v>
       </c>
@@ -2937,10 +2928,10 @@
       <c r="B2" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="C2" s="31">
+      <c r="C2" s="25">
         <v>33.996805000000002</v>
       </c>
-      <c r="D2" s="32">
+      <c r="D2" s="26">
         <v>71.440115000000006</v>
       </c>
       <c r="E2" s="16">
@@ -2951,11 +2942,11 @@
         <f t="shared" ref="F2" si="1">(E2*6)-183</f>
         <v>69</v>
       </c>
-      <c r="G2" s="34">
+      <c r="G2" s="28">
         <f t="shared" ref="G2" si="2">500000 + 0.9996 * (6378137/SQRT(1-0.00669438*(SIN(RADIANS(C2))^2))) * ((RADIANS(D2-F2)*COS(RADIANS(C2))) + (1 - TAN(RADIANS(C2))^2 + 0.0067395*(COS(RADIANS(C2))^2)) * ((RADIANS(D2-F2)*COS(RADIANS(C2)))^3)/6 + (5 - 18*TAN(RADIANS(C2))^2 + TAN(RADIANS(C2))^4 + 72*0.0067395*(COS(RADIANS(C2))^2) - 58*0.0067395) * ((RADIANS(D2-F2)*COS(RADIANS(C2)))^5)/120)</f>
         <v>725373.50020119664</v>
       </c>
-      <c r="H2" s="34">
+      <c r="H2" s="28">
         <f t="shared" ref="H2" si="3">0.9996 * ((6378137*(0.9983242984*RADIANS(C2) - 0.002514607*SIN(2*RADIANS(C2)) + 0.000002639*SIN(4*RADIANS(C2)) - 0.000000003*SIN(6*RADIANS(C2)))) + (6378137/SQRT(1-0.00669438*(SIN(RADIANS(C2))^2))) * TAN(RADIANS(C2)) * (((RADIANS(D2-F2)*COS(RADIANS(C2)))^2)/2 + (5 - TAN(RADIANS(C2))^2 + 9*0.0067395*(COS(RADIANS(C2))^2) + 4*(0.0067395*(COS(RADIANS(C2))^2))^2) * ((RADIANS(D2-F2)*COS(RADIANS(C2)))^4)/24 + (61 - 58*TAN(RADIANS(C2))^2 + TAN(RADIANS(C2))^4 + 600*0.0067395*(COS(RADIANS(C2))^2) - 330*0.0067395) * ((RADIANS(D2-F2)*COS(RADIANS(C2)))^6)/720))</f>
         <v>3764486.0991854998</v>
       </c>
@@ -2971,10 +2962,10 @@
       <c r="B3" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="C3" s="31">
+      <c r="C3" s="25">
         <v>33.996749999999999</v>
       </c>
-      <c r="D3" s="32">
+      <c r="D3" s="26">
         <v>71.440866</v>
       </c>
       <c r="E3" s="16">
@@ -2985,11 +2976,11 @@
         <f t="shared" ref="F3:F13" si="6">(E3*6)-183</f>
         <v>69</v>
       </c>
-      <c r="G3" s="34">
+      <c r="G3" s="28">
         <f t="shared" ref="G3:G13" si="7">500000 + 0.9996 * (6378137/SQRT(1-0.00669438*(SIN(RADIANS(C3))^2))) * ((RADIANS(D3-F3)*COS(RADIANS(C3))) + (1 - TAN(RADIANS(C3))^2 + 0.0067395*(COS(RADIANS(C3))^2)) * ((RADIANS(D3-F3)*COS(RADIANS(C3)))^3)/6 + (5 - 18*TAN(RADIANS(C3))^2 + TAN(RADIANS(C3))^4 + 72*0.0067395*(COS(RADIANS(C3))^2) - 58*0.0067395) * ((RADIANS(D3-F3)*COS(RADIANS(C3)))^5)/120)</f>
         <v>725443.02518306125</v>
       </c>
-      <c r="H3" s="34">
+      <c r="H3" s="28">
         <f t="shared" ref="H3:H13" si="8">0.9996 * ((6378137*(0.9983242984*RADIANS(C3) - 0.002514607*SIN(2*RADIANS(C3)) + 0.000002639*SIN(4*RADIANS(C3)) - 0.000000003*SIN(6*RADIANS(C3)))) + (6378137/SQRT(1-0.00669438*(SIN(RADIANS(C3))^2))) * TAN(RADIANS(C3)) * (((RADIANS(D3-F3)*COS(RADIANS(C3)))^2)/2 + (5 - TAN(RADIANS(C3))^2 + 9*0.0067395*(COS(RADIANS(C3))^2) + 4*(0.0067395*(COS(RADIANS(C3))^2))^2) * ((RADIANS(D3-F3)*COS(RADIANS(C3)))^4)/24 + (61 - 58*TAN(RADIANS(C3))^2 + TAN(RADIANS(C3))^4 + 600*0.0067395*(COS(RADIANS(C3))^2) - 330*0.0067395) * ((RADIANS(D3-F3)*COS(RADIANS(C3)))^6)/720))</f>
         <v>3764481.6522049252</v>
       </c>
@@ -3005,10 +2996,10 @@
       <c r="B4" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="C4" s="31">
+      <c r="C4" s="25">
         <v>33.996701999999999</v>
       </c>
-      <c r="D4" s="32">
+      <c r="D4" s="26">
         <v>71.441635000000005</v>
       </c>
       <c r="E4" s="16">
@@ -3019,11 +3010,11 @@
         <f t="shared" si="6"/>
         <v>69</v>
       </c>
-      <c r="G4" s="34">
+      <c r="G4" s="28">
         <f t="shared" si="7"/>
         <v>725514.19465295249</v>
       </c>
-      <c r="H4" s="34">
+      <c r="H4" s="28">
         <f t="shared" si="8"/>
         <v>3764478.021790558</v>
       </c>
@@ -3039,10 +3030,10 @@
       <c r="B5" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="C5" s="31">
+      <c r="C5" s="25">
         <v>33.996651</v>
       </c>
-      <c r="D5" s="32">
+      <c r="D5" s="26">
         <v>71.442519000000004</v>
       </c>
       <c r="E5" s="16">
@@ -3053,11 +3044,11 @@
         <f t="shared" si="6"/>
         <v>69</v>
       </c>
-      <c r="G5" s="34">
+      <c r="G5" s="28">
         <f t="shared" si="7"/>
         <v>725595.99621613557</v>
       </c>
-      <c r="H5" s="34">
+      <c r="H5" s="28">
         <f t="shared" si="8"/>
         <v>3764474.3125480362</v>
       </c>
@@ -3073,10 +3064,10 @@
       <c r="B6" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="C6" s="31">
+      <c r="C6" s="25">
         <v>33.996628999999999</v>
       </c>
-      <c r="D6" s="32">
+      <c r="D6" s="26">
         <v>71.442920000000001</v>
       </c>
       <c r="E6" s="16">
@@ -3087,11 +3078,11 @@
         <f t="shared" si="6"/>
         <v>69</v>
       </c>
-      <c r="G6" s="34">
+      <c r="G6" s="28">
         <f t="shared" si="7"/>
         <v>725633.10007064731</v>
       </c>
-      <c r="H6" s="34">
+      <c r="H6" s="28">
         <f t="shared" si="8"/>
         <v>3764472.7560407557</v>
       </c>
@@ -3107,10 +3098,10 @@
       <c r="B7" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="C7" s="31">
+      <c r="C7" s="25">
         <v>33.996603999999998</v>
       </c>
-      <c r="D7" s="32">
+      <c r="D7" s="26">
         <v>71.443309999999997</v>
       </c>
       <c r="E7" s="16">
@@ -3121,11 +3112,11 @@
         <f t="shared" si="6"/>
         <v>69</v>
       </c>
-      <c r="G7" s="34">
+      <c r="G7" s="28">
         <f t="shared" si="7"/>
         <v>725669.19567195559</v>
       </c>
-      <c r="H7" s="34">
+      <c r="H7" s="28">
         <f t="shared" si="8"/>
         <v>3764470.842684621</v>
       </c>
@@ -3141,10 +3132,10 @@
       <c r="B8" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="C8" s="31">
+      <c r="C8" s="25">
         <v>33.996184</v>
       </c>
-      <c r="D8" s="32">
+      <c r="D8" s="26">
         <v>71.443397000000004</v>
       </c>
       <c r="E8" s="16">
@@ -3155,11 +3146,11 @@
         <f t="shared" si="6"/>
         <v>69</v>
       </c>
-      <c r="G8" s="34">
+      <c r="G8" s="28">
         <f t="shared" si="7"/>
         <v>725678.34449331742</v>
       </c>
-      <c r="H8" s="34">
+      <c r="H8" s="28">
         <f t="shared" si="8"/>
         <v>3764424.449714717</v>
       </c>
@@ -3175,10 +3166,10 @@
       <c r="B9" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="C9" s="31">
+      <c r="C9" s="25">
         <v>33.995657999999999</v>
       </c>
-      <c r="D9" s="32">
+      <c r="D9" s="26">
         <v>71.443360999999996</v>
       </c>
       <c r="E9" s="16">
@@ -3189,11 +3180,11 @@
         <f t="shared" si="6"/>
         <v>69</v>
       </c>
-      <c r="G9" s="34">
+      <c r="G9" s="28">
         <f t="shared" si="7"/>
         <v>725676.41064086824</v>
       </c>
-      <c r="H9" s="34">
+      <c r="H9" s="28">
         <f t="shared" si="8"/>
         <v>3764366.0285358168</v>
       </c>
@@ -3209,10 +3200,10 @@
       <c r="B10" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="C10" s="31">
+      <c r="C10" s="25">
         <v>33.995655999999997</v>
       </c>
-      <c r="D10" s="32">
+      <c r="D10" s="26">
         <v>71.443374000000006</v>
       </c>
       <c r="E10" s="16">
@@ -3223,11 +3214,11 @@
         <f t="shared" si="6"/>
         <v>69</v>
       </c>
-      <c r="G10" s="34">
+      <c r="G10" s="28">
         <f t="shared" si="7"/>
         <v>725677.61692872411</v>
       </c>
-      <c r="H10" s="34">
+      <c r="H10" s="28">
         <f t="shared" si="8"/>
         <v>3764365.8353578378</v>
       </c>
@@ -3243,10 +3234,10 @@
       <c r="B11" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="C11" s="31">
+      <c r="C11" s="25">
         <v>33.995666999999997</v>
       </c>
-      <c r="D11" s="32">
+      <c r="D11" s="26">
         <v>71.443359999999998</v>
       </c>
       <c r="E11" s="16">
@@ -3257,11 +3248,11 @@
         <f t="shared" si="6"/>
         <v>69</v>
       </c>
-      <c r="G11" s="34">
+      <c r="G11" s="28">
         <f t="shared" si="7"/>
         <v>725676.29443998355</v>
       </c>
-      <c r="H11" s="34">
+      <c r="H11" s="28">
         <f t="shared" si="8"/>
         <v>3764367.0245758388</v>
       </c>
@@ -3277,10 +3268,10 @@
       <c r="B12" s="17" t="s">
         <v>75</v>
       </c>
-      <c r="C12" s="31">
+      <c r="C12" s="25">
         <v>33.995356000000001</v>
       </c>
-      <c r="D12" s="32">
+      <c r="D12" s="26">
         <v>71.443335000000005</v>
       </c>
       <c r="E12" s="16">
@@ -3291,11 +3282,11 @@
         <f t="shared" si="6"/>
         <v>69</v>
       </c>
-      <c r="G12" s="34">
+      <c r="G12" s="28">
         <f t="shared" si="7"/>
         <v>725674.80781942757</v>
       </c>
-      <c r="H12" s="34">
+      <c r="H12" s="28">
         <f t="shared" si="8"/>
         <v>3764332.474591224</v>
       </c>
@@ -3491,71 +3482,71 @@
       <c r="A16" s="24" t="s">
         <v>128</v>
       </c>
-      <c r="B16" s="27" t="s">
+      <c r="B16" s="37" t="s">
         <v>129</v>
       </c>
-      <c r="C16" s="26"/>
-      <c r="D16" s="26"/>
+      <c r="C16" s="36"/>
+      <c r="D16" s="36"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="B17" s="28" t="s">
+      <c r="B17" s="38" t="s">
         <v>131</v>
       </c>
-      <c r="C17" s="29"/>
-      <c r="D17" s="29"/>
+      <c r="C17" s="39"/>
+      <c r="D17" s="39"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B18" s="28" t="s">
+      <c r="B18" s="38" t="s">
         <v>132</v>
       </c>
-      <c r="C18" s="29"/>
-      <c r="D18" s="29"/>
+      <c r="C18" s="39"/>
+      <c r="D18" s="39"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="B19" s="28" t="s">
+      <c r="B19" s="38" t="s">
         <v>134</v>
       </c>
-      <c r="C19" s="29"/>
-      <c r="D19" s="29"/>
+      <c r="C19" s="39"/>
+      <c r="D19" s="39"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="B20" s="28" t="s">
+      <c r="B20" s="38" t="s">
         <v>136</v>
       </c>
-      <c r="C20" s="29"/>
-      <c r="D20" s="29"/>
+      <c r="C20" s="39"/>
+      <c r="D20" s="39"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="B21" s="28" t="s">
+      <c r="B21" s="38" t="s">
         <v>138</v>
       </c>
-      <c r="C21" s="29"/>
-      <c r="D21" s="29"/>
+      <c r="C21" s="39"/>
+      <c r="D21" s="39"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="B22" s="28" t="s">
+      <c r="B22" s="38" t="s">
         <v>140</v>
       </c>
-      <c r="C22" s="29"/>
-      <c r="D22" s="29"/>
+      <c r="C22" s="39"/>
+      <c r="D22" s="39"/>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>